<commit_message>
Clean run across all four names after the credit top-up
Every company healthy this time: HD, ADI and DE at nine of nine lenses surviving
with every citation verified, Hays at seven of nine. The health guard confirms
all four workbooks took their numbers from a healthy run, with no degraded run
used anywhere.

Deere is back where it should be. Its previous figures came from the run where
the API ran out mid-flight, and were the consensus figure showing through the
positioning fallback rather than a forecast at all.

The baseline panel comes off the forecast sheet, since the baseline itself is
gone from the results.

Twelve numbers, all four workbooks verified, architecture sealed at 0.32 MB with
no external reference.
</commit_message>
<xml_diff>
--- a/submission/ADI-FY2026Q3.xlsx
+++ b/submission/ADI-FY2026Q3.xlsx
@@ -581,7 +581,7 @@
         <x:v>USDm</x:v>
       </x:c>
       <x:c r="C7" s="34">
-        <x:v>3932</x:v>
+        <x:v>3930</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="29" customHeight="1">
@@ -592,7 +592,7 @@
         <x:v>USD / share</x:v>
       </x:c>
       <x:c r="C8" s="35">
-        <x:v>3.355</x:v>
+        <x:v>3.35</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="29" customHeight="1">
@@ -603,7 +603,7 @@
         <x:v>%</x:v>
       </x:c>
       <x:c r="C9" s="36">
-        <x:v>73</x:v>
+        <x:v>73.1</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">

</xml_diff>

<commit_message>
Record the 17:15 final run, all four forecast fresh
Run 3083d3e5. Four companies, no failures, no retries, $6.01 of the $25
ceiling. Exit code 0 -- every number forecast in this run rather than carried
forward.

The 16:13Z attempt is kept alongside it. That one failed all four on a missing
ANTHROPIC_API_KEY and fell back to the previous workbooks, which is what exit
code 2 is for and why the log of a failed attempt is worth as much as this one.

DE moved most against the 14:10Z run: revenue 12470 -> 11850 and P&PA operating
profit 560 -> 570. HAS left stage D degraded with two metrics projected and the
judge recovered the third, so all twelve cells are populated.

runs/ stays untracked as before; the log records each results.json path.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/submission/ADI-FY2026Q3.xlsx
+++ b/submission/ADI-FY2026Q3.xlsx
@@ -581,7 +581,7 @@
         <x:v>USDm</x:v>
       </x:c>
       <x:c r="C7" s="34">
-        <x:v>3930</x:v>
+        <x:v>3958</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="29" customHeight="1">
@@ -592,7 +592,7 @@
         <x:v>USD / share</x:v>
       </x:c>
       <x:c r="C8" s="35">
-        <x:v>3.35</x:v>
+        <x:v>3.4</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="29" customHeight="1">

</xml_diff>